<commit_message>
feat: data validation in Excel, incomplete student warnings, 1º-2º Primaria support
- Excel data validation: dropdowns for Centro ERG, Conservatorio, Curso Cons.,
  Especialidad, Curso ERG and Tipo centro from reference sheets
- New "Listas" sheet with all valid courses and 33 specialties
- Validation ranges support up to 100 centers, 50 conservatories, 500 students
- Students missing Curso Conservatorio or Curso ERG show a warning and are
  excluded from cards view (still visible in table view)
- Added 1º and 2º Primaria to ERG course index for advanced students
- Export PDF button moved into summary bar
- Contact email added to footer

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ejemplo_coordinacion.xlsx
+++ b/ejemplo_coordinacion.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Centros" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Conservatorios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Alumnado" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Listas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Alumnado" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001A1A2E"/>
         <bgColor rgb="001A1A2E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004361EE"/>
+        <bgColor rgb="004361EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +71,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -737,6 +747,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Tipo de centro" prompt="CEIP o IES" type="list">
+      <formula1>"CEIP,IES"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -750,7 +765,7 @@
   <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
@@ -929,6 +944,383 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cursos Conservatorio</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Cursos ERG</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Especialidades</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1º EEM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1º Primaria</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DANZA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2º EEM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2º Primaria</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DANZA CLÁSICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3º EEM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3º Primaria</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DANZA CONTEMPORÁNEA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4º EEM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4º Primaria</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DANZA ESPAÑOLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1º EPM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5º Primaria</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ACORDEÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2º EPM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6º Primaria</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ARPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3º EPM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1º ESO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BAJO ELÉCTRICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4º EPM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2º ESO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CANTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5º EPM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3º ESO</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CANTO VALENCIANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6º EPM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>4º ESO</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CLARINETE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1º Bachillerato</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CLAVECÍN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2º Bachillerato</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CONTRABAJO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DULZAINA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FAGOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FLAUTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FLAUTA DE PICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>GUITARRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>GUITARRA ELÉCTRICA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>INSTRUMENTOS DE CUERDA PULSADA DEL RENACIMIENTO Y BARROCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>INSTRUMENTOS DE PLECTRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OBOE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ÓRGANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PERCUSIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PIANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>SAXOFÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>TROMBÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>TROMPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>TROMPETA</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TUBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>VIOLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>VIOLA DA GAMBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>VIOLÍN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>VIOLONCHELO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -936,16 +1328,16 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="35" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1053,7 +1445,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1125,7 +1517,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1193,7 +1585,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1261,12 +1653,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>3º Primaria</t>
+          <t>2º Primaria</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1286,12 +1678,12 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Sandra Molina</t>
+          <t>Carlos Vera</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>s.molina@edu.gva.es</t>
+          <t>c.vera@edu.gva.es</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr"/>
@@ -1329,7 +1721,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1401,7 +1793,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1416,12 +1808,12 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Marcos Iborra</t>
+          <t>Elena Pascual</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>m.iborra@consdanza.es</t>
+          <t>e.pascual@consdanza.es</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1434,11 +1826,7 @@
           <t>r.ibanez@edu.gva.es</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Familia solicita reunión con ambos tutores</t>
-        </is>
-      </c>
+      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1448,12 +1836,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Moreno Garrido</t>
+          <t>Sánchez Lozano</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Enrique</t>
+          <t>Raúl</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1463,7 +1851,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Conservatorio Profesional de Danza</t>
+          <t>Conservatorio Municipal de Música</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1473,7 +1861,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1488,12 +1876,12 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Marcos Iborra</t>
+          <t>Pilar Esteve</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>m.iborra@consdanza.es</t>
+          <t>p.esteve@consmmusica.es</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1541,7 +1929,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1613,7 +2001,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1681,7 +2069,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>DANZA CONTEMPORÁNEA</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1753,12 +2141,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>3º Primaria</t>
+          <t>2º Primaria</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1778,12 +2166,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Sandra Molina</t>
+          <t>Carlos Vera</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>s.molina@edu.gva.es</t>
+          <t>c.vera@edu.gva.es</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1821,7 +2209,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1893,7 +2281,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1961,7 +2349,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>DANZA CONTEMPORÁNEA</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -2029,7 +2417,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -2101,7 +2489,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -2169,7 +2557,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2237,7 +2625,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2305,7 +2693,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2369,7 +2757,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2441,7 +2829,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2509,7 +2897,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2577,7 +2965,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2649,7 +3037,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2717,12 +3105,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>3º Primaria</t>
+          <t>2º Primaria</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2742,12 +3130,12 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Marta Pons</t>
+          <t>Pablo Sanz</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>m.pons@edu.gva.es</t>
+          <t>p.sanz@edu.gva.es</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr"/>
@@ -2785,12 +3173,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>3º Primaria</t>
+          <t>1º Primaria</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2810,12 +3198,12 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Marta Pons</t>
+          <t>Inés Roig</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>m.pons@edu.gva.es</t>
+          <t>i.roig@edu.gva.es</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr"/>
@@ -2853,7 +3241,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>VIOLONCHELO</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2921,7 +3309,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2993,12 +3381,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>3º Primaria</t>
+          <t>2º Primaria</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3018,12 +3406,12 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Marta Pons</t>
+          <t>Pablo Sanz</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>m.pons@edu.gva.es</t>
+          <t>p.sanz@edu.gva.es</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr"/>
@@ -3061,7 +3449,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3133,7 +3521,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3201,7 +3589,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -3269,7 +3657,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3337,12 +3725,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>6º Primaria</t>
+          <t>5º Primaria</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3352,22 +3740,22 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Elena Pascual</t>
+          <t>Silvia Arnau</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>e.pascual@consdanza.es</t>
+          <t>s.arnau@consdanza.es</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Diego Soriano</t>
+          <t>Lucía Ferrer</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>d.soriano@edu.gva.es</t>
+          <t>l.ferrer@edu.gva.es</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr"/>
@@ -3380,12 +3768,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Moreno Jiménez</t>
+          <t>Vidal Moreno</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Bruno</t>
+          <t>Diego</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3405,7 +3793,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3415,7 +3803,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Plurilingüe/Mañana</t>
+          <t>Ordinaria/Mañana</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -3453,7 +3841,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Bruno</t>
+          <t>Eva</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -3463,7 +3851,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Conservatorio Profesional de Danza</t>
+          <t>Conservatorio Municipal de Música</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3473,7 +3861,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3488,12 +3876,12 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Silvia Arnau</t>
+          <t>Pilar Esteve</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>s.arnau@consdanza.es</t>
+          <t>p.esteve@consmmusica.es</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3545,7 +3933,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3613,7 +4001,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3681,7 +4069,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3749,7 +4137,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3817,7 +4205,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3877,7 +4265,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3949,7 +4337,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -4021,7 +4409,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -4089,7 +4477,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4161,7 +4549,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -4229,7 +4617,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4301,7 +4689,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4369,7 +4757,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4437,7 +4825,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -4505,17 +4893,17 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>3º ESO</t>
+          <t>2º ESO</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Ordinaria/Tarde</t>
+          <t>Ordinaria/Mañana</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -4530,12 +4918,12 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Amparo Llorens</t>
+          <t>Manuel Ribera</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>a.llorens@edu.gva.es</t>
+          <t>m.ribera@edu.gva.es</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr"/>
@@ -4553,7 +4941,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Inés</t>
+          <t>Sara</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -4573,7 +4961,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4641,7 +5029,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4709,7 +5097,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -4769,7 +5157,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -4837,7 +5225,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4905,7 +5293,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -4977,7 +5365,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -5045,7 +5433,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -5113,7 +5501,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -5181,7 +5569,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -5249,7 +5637,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5317,7 +5705,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -5385,7 +5773,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>DANZA CONTEMPORÁNEA</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -5453,7 +5841,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -5521,7 +5909,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -5589,7 +5977,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>DANZA CONTEMPORÁNEA</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -5657,7 +6045,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -5725,7 +6113,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -5797,7 +6185,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -5865,7 +6253,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -5933,7 +6321,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -6001,7 +6389,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -6069,7 +6457,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -6141,7 +6529,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -6209,7 +6597,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -6281,7 +6669,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Clarinete</t>
+          <t>CLARINETE</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -6349,7 +6737,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -6417,7 +6805,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -6477,7 +6865,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -6545,7 +6933,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>VIOLONCHELO</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -6613,7 +7001,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -6681,7 +7069,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -6749,7 +7137,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -6764,12 +7152,12 @@
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>Elena Pascual</t>
+          <t>Marcos Iborra</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>e.pascual@consdanza.es</t>
+          <t>m.iborra@consdanza.es</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
@@ -6782,7 +7170,11 @@
           <t>v.crespo@edu.gva.es</t>
         </is>
       </c>
-      <c r="N85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Posible cambio de centro ERG el próximo curso</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6817,7 +7209,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -6885,7 +7277,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -6953,7 +7345,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>VIOLONCHELO</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -7021,7 +7413,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -7089,7 +7481,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -7157,7 +7549,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Flauta travesera</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -7217,7 +7609,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>PERCUSIÓN</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -7289,7 +7681,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -7357,7 +7749,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -7425,7 +7817,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>DANZA CONTEMPORÁNEA</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -7497,7 +7889,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -7569,7 +7961,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -7637,7 +8029,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -7705,7 +8097,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -7777,7 +8169,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -7845,7 +8237,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -7913,7 +8305,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Guitarra</t>
+          <t>GUITARRA</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -7981,44 +8373,40 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>1º Bachillerato</t>
+          <t>2º Bachillerato</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>Plurilingüe/Mañana</t>
+          <t>Ordinaria/Mañana</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
         <is>
-          <t>Silvia Arnau</t>
+          <t>Elena Pascual</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>s.arnau@consdanza.es</t>
+          <t>e.pascual@consdanza.es</t>
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
-          <t>Irene Campos</t>
+          <t>Fernando Aguilar</t>
         </is>
       </c>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>i.campos@edu.gva.es</t>
-        </is>
-      </c>
-      <c r="N103" s="2" t="inlineStr">
-        <is>
-          <t>Necesita coordinación especial: sale 15 min antes del IES</t>
-        </is>
-      </c>
+          <t>f.aguilar@edu.gva.es</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -8028,12 +8416,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Santos Ramírez</t>
+          <t>Molina Santos</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Javier</t>
+          <t>Eva</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -8053,12 +8441,12 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Violín</t>
+          <t>VIOLONCHELO</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>1º Bachillerato</t>
+          <t>4º ESO</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -8068,22 +8456,22 @@
       </c>
       <c r="J104" s="2" t="inlineStr">
         <is>
-          <t>Antonio Grau</t>
+          <t>Ángel Fuster</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>a.grau@consmmusica.es</t>
+          <t>a.fuster@consmmusica.es</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
-          <t>Irene Campos</t>
+          <t>Tomás Gil</t>
         </is>
       </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>i.campos@edu.gva.es</t>
+          <t>t.gil@edu.gva.es</t>
         </is>
       </c>
       <c r="N104" s="2" t="inlineStr"/>
@@ -8096,12 +8484,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Cortés Blanco</t>
+          <t>Gil Cortés</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Marcos</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -8121,42 +8509,42 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>OBOE</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>2º Bachillerato</t>
+          <t>1º Bachillerato</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Ordinaria/Mañana</t>
+          <t>Ordinaria/Tarde</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
         <is>
-          <t>Ángel Fuster</t>
+          <t>Gonzalo Herrero</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>a.fuster@consmmusica.es</t>
+          <t>g.herrero@consmmusica.es</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
-          <t>Fernando Aguilar</t>
+          <t>Irene Campos</t>
         </is>
       </c>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>f.aguilar@edu.gva.es</t>
+          <t>i.campos@edu.gva.es</t>
         </is>
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>Repetidor/a en ERG, primer año en conservatorio</t>
+          <t>Solicita adaptación horaria por desplazamiento entre centros</t>
         </is>
       </c>
     </row>
@@ -8168,12 +8556,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Castro Bou</t>
+          <t>Guerrero Torres</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Marta</t>
+          <t>Héctor</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -8193,12 +8581,12 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>DANZA ESPAÑOLA</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>1º Bachillerato</t>
+          <t>2º Bachillerato</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -8218,12 +8606,12 @@
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>Irene Campos</t>
+          <t>Fernando Aguilar</t>
         </is>
       </c>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>i.campos@edu.gva.es</t>
+          <t>f.aguilar@edu.gva.es</t>
         </is>
       </c>
       <c r="N106" s="2" t="inlineStr"/>
@@ -8236,12 +8624,12 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Hernández Blanco</t>
+          <t>Bou Marín</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Claudia</t>
+          <t>Ana</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -8261,7 +8649,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Trompeta</t>
+          <t>VIOLÍN</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
@@ -8271,17 +8659,17 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>Plurilingüe/Mañana</t>
+          <t>Ordinaria/Mañana</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
         <is>
-          <t>Ángel Fuster</t>
+          <t>Isabel Romero</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>a.fuster@consmmusica.es</t>
+          <t>i.romero@consmmusica.es</t>
         </is>
       </c>
       <c r="L107" s="2" t="inlineStr">
@@ -8304,12 +8692,12 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Marín Guerrero</t>
+          <t>Garrido Suárez</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Lucía</t>
+          <t>Gonzalo</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -8329,17 +8717,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Oboe</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>2º Bachillerato</t>
+          <t>4º ESO</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>Ordinaria/Mañana</t>
+          <t>Ordinaria/Tarde</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -8354,12 +8742,12 @@
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>Fernando Aguilar</t>
+          <t>Tomás Gil</t>
         </is>
       </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>f.aguilar@edu.gva.es</t>
+          <t>t.gil@edu.gva.es</t>
         </is>
       </c>
       <c r="N108" s="2" t="inlineStr"/>
@@ -8372,12 +8760,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Rodríguez Ramírez</t>
+          <t>Ramírez Navarro</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Cristina</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -8397,7 +8785,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>TROMPETA</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -8407,17 +8795,17 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>Ordinaria/Mañana</t>
+          <t>Ordinaria/Tarde</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>Tomás Ripoll</t>
+          <t>Ángel Fuster</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>t.ripoll@consmmusica.es</t>
+          <t>a.fuster@consmmusica.es</t>
         </is>
       </c>
       <c r="L109" s="2" t="inlineStr">
@@ -8430,7 +8818,11 @@
           <t>f.aguilar@edu.gva.es</t>
         </is>
       </c>
-      <c r="N109" s="2" t="inlineStr"/>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>Alumno/a con NEE: adaptación curricular en ERG</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -8440,12 +8832,12 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Navarro Lozano</t>
+          <t>Molina Soler</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -8465,12 +8857,12 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Piano</t>
+          <t>DANZA CLÁSICA</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>1º Bachillerato</t>
+          <t>2º Bachillerato</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
@@ -8490,15 +8882,19 @@
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>Irene Campos</t>
+          <t>Fernando Aguilar</t>
         </is>
       </c>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>i.campos@edu.gva.es</t>
-        </is>
-      </c>
-      <c r="N110" s="2" t="inlineStr"/>
+          <t>f.aguilar@edu.gva.es</t>
+        </is>
+      </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>Necesita coordinación especial: sale 15 min antes del IES</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -8508,12 +8904,12 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Santos Navarro</t>
+          <t>Pla Vidal</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Teresa</t>
+          <t>Pablo</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -8533,12 +8929,12 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Saxofón</t>
+          <t>FLAUTA</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>4º ESO</t>
+          <t>2º Bachillerato</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -8548,22 +8944,22 @@
       </c>
       <c r="J111" s="2" t="inlineStr">
         <is>
-          <t>Gonzalo Herrero</t>
+          <t>Pilar Esteve</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>g.herrero@consmmusica.es</t>
+          <t>p.esteve@consmmusica.es</t>
         </is>
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>Tomás Gil</t>
+          <t>Fernando Aguilar</t>
         </is>
       </c>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>t.gil@edu.gva.es</t>
+          <t>f.aguilar@edu.gva.es</t>
         </is>
       </c>
       <c r="N111" s="2" t="inlineStr"/>
@@ -8576,12 +8972,12 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Díaz Hernández</t>
+          <t>Pla Díaz</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Marcos</t>
+          <t>Andrés</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -8601,12 +8997,12 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Percusión</t>
+          <t>SAXOFÓN</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>1º Bachillerato</t>
+          <t>2º Bachillerato</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -8616,22 +9012,22 @@
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>Tomás Ripoll</t>
+          <t>Gonzalo Herrero</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>t.ripoll@consmmusica.es</t>
+          <t>g.herrero@consmmusica.es</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>Irene Campos</t>
+          <t>Fernando Aguilar</t>
         </is>
       </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>i.campos@edu.gva.es</t>
+          <t>f.aguilar@edu.gva.es</t>
         </is>
       </c>
       <c r="N112" s="2" t="inlineStr"/>
@@ -8644,12 +9040,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Vidal Cortés</t>
+          <t>López Hernández</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Natalia</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -8669,46 +9065,59 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Violonchelo</t>
+          <t>PIANO</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>2º Bachillerato</t>
+          <t>1º Bachillerato</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>Ordinaria/Tarde</t>
+          <t>Ordinaria/Mañana</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
         <is>
-          <t>Ángel Fuster</t>
+          <t>Francisco Pérez</t>
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>a.fuster@consmmusica.es</t>
+          <t>f.perez@consmmusica.es</t>
         </is>
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>Fernando Aguilar</t>
+          <t>Irene Campos</t>
         </is>
       </c>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>f.aguilar@edu.gva.es</t>
-        </is>
-      </c>
-      <c r="N113" s="2" t="inlineStr">
-        <is>
-          <t>Posible cambio de centro ERG el próximo curso</t>
-        </is>
-      </c>
+          <t>i.campos@edu.gva.es</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="5">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Centro no válido" error="Selecciona un centro de la hoja Centros" promptTitle="Centro ERG" prompt="Selecciona el centro ERG del alumno/a" type="list">
+      <formula1>=Centros!$B$2:$B$101</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Conservatorio no válido" error="Selecciona un conservatorio de la hoja Conservatorios" promptTitle="Conservatorio" prompt="Selecciona el conservatorio del alumno/a" type="list">
+      <formula1>=Conservatorios!$A$2:$A$51</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Curso no válido" error="Selecciona un curso de conservatorio válido" promptTitle="Curso Conservatorio" prompt="Selecciona el curso del conservatorio" type="list">
+      <formula1>=Listas!$A$2:$A$11</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Especialidad no válida" error="Selecciona una especialidad de la lista" promptTitle="Especialidad" prompt="Selecciona la especialidad" type="list">
+      <formula1>=Listas!$C$2:$C$34</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Curso ERG no válido" error="Selecciona un curso ERG válido" promptTitle="Curso ERG" prompt="Selecciona el curso en el centro ERG" type="list">
+      <formula1>=Listas!$B$2:$B$13</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>